<commit_message>
Fix header nav lookup on AEM author, public image URLs, site paths mapping
- header: resolve nav from the page's AEM site root (/content/<site>/nav) before
  /content/nav and /nav, so the header renders in Universal Editor
- importer: page and nav images point at the public code bus so AEM can ingest them
- paths.json: map /content/innovationlabgt/ to the site root

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -67,7 +67,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-09-29T20:27:01.361Z</t>
+    <t>2026-09-29T21:03:36.050Z</t>
   </si>
   <si>
     <t>http://127.0.0.1:8765/nav.html</t>
@@ -82,7 +82,7 @@
     <t>innovationlabgt/bronco</t>
   </si>
   <si>
-    <t>2026-09-29T20:16:57.195Z</t>
+    <t>2026-09-29T21:03:29.578Z</t>
   </si>
 </sst>
 </file>

</xml_diff>